<commit_message>
Update basic app forms
</commit_message>
<xml_diff>
--- a/basic-forms/forms/app/comparing_values.xlsx
+++ b/basic-forms/forms/app/comparing_values.xlsx
@@ -1,8 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <fileVersion appName="Calc" lowestEdited="5"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
@@ -10,20 +10,21 @@
   <sheets>
     <sheet name="survey" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="settings" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="chtx" sheetId="3" state="hidden" r:id="rId5"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
+      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
   <authors>
-    <author>Unknown Author</author>
+    <author>Author</author>
   </authors>
   <commentList>
     <comment ref="A1" authorId="0">
@@ -35,20 +36,30 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">Determines what kinds of values are allowed and how the field is displayed. For certain types, further customization is possible using the appearance and parameters columns.
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF0000FF"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">https://docs.getodk.org/form-question-types/
-</t>
+https://docs.getodk.org/form-question-types/</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>6</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>2</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="B1" authorId="0">
       <text>
@@ -61,6 +72,27 @@
           <t xml:space="preserve">Variable name. It may not contain spaces and must start with a letter or underscore. You should use a short, descriptive name and can use underscores to separate words. For example: date_of_birth.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>2</xdr:col>
+                <xdr:colOff>6</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>4</xdr:col>
+                <xdr:colOff>2</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="C1" authorId="0">
       <text>
@@ -74,6 +106,27 @@
 Can be translated.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>6</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>5</xdr:col>
+                <xdr:colOff>2</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="D1" authorId="0">
       <text>
@@ -87,6 +140,27 @@
 Can be translated.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>4</xdr:col>
+                <xdr:colOff>6</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>6</xdr:col>
+                <xdr:colOff>2</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="E1" authorId="0">
       <text>
@@ -97,9 +171,30 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">An expression that determines whether a question will be displayed to a user or not. Lets you define branching or skip logic. 
-https://docs.getodk.org/form-logic/#conditionally-showing-questions</t>
+See the Relevance tab for examples.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>5</xdr:col>
+                <xdr:colOff>6</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>7</xdr:col>
+                <xdr:colOff>2</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="F1" authorId="0">
       <text>
@@ -113,6 +208,27 @@
 These can be specific to the field type.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>6</xdr:col>
+                <xdr:colOff>6</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>8</xdr:col>
+                <xdr:colOff>21</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="G1" authorId="0">
       <text>
@@ -123,32 +239,41 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">An expression that will be evaluated to determine the value of the field.
-⚠️ Expressions may be re-evaluated at any time. 
-To limit when expressions are evaluated, for example to specify dynamic defaults use the once() function. 
+Expressions may be re-evaluated at any time. Question types with calculations should be marked as read-only. Otherwise, a user-provided value may be replaced by a calculated one.
+To limit when expressions are evaluated, for example to specify dynamic defaults, use the trigger column or the once() function. 
 https://docs.getodk.org/form-logic/#when-expressions-are-evaluated</t>
         </r>
       </text>
-    </comment>
-    <comment ref="H1" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Can include a human-friendly note to describe the row. This will be ignored by all ODK tools.</t>
-        </r>
-      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>7</xdr:col>
+                <xdr:colOff>6</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>9</xdr:col>
+                <xdr:colOff>21</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
   <authors>
-    <author>Unknown Author</author>
+    <author>Author</author>
   </authors>
   <commentList>
     <comment ref="A1" authorId="0">
@@ -163,6 +288,27 @@
 https://docs.getodk.org/xlsform/#the-settings-sheet</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>6</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>2</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="B1" authorId="0">
       <text>
@@ -173,9 +319,32 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">The unique version code that identifies the current state of the form. A common convention is to use a format like yyyymmddrr. For example, 2017021501 is the 1st revision from Feb 15th, 2017.
-By default, this template uses a formula to create a date-based version that will update automatically.</t>
+A formula can be used to update the version automatically: `=TEXT(NOW(), "yyyymmddhhmmss")`
+This `version` is recorded in the form xml and is primarily useful for determining which version of the xlsform was used to produce the xml. A separate `form_version` property is generated for each form when it is uploaded to the CHT server. This is the version set on report docs produced by the form.
+https://docs.communityhealthtoolkit.org/building/forms/versioning/</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>2</xdr:col>
+                <xdr:colOff>6</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>4</xdr:col>
+                <xdr:colOff>2</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="C1" authorId="0">
       <text>
@@ -185,9 +354,32 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Set to ‘pages’ to indicate that groups with the `field-list` appearance represent separate form pages (and all other questions will be shown on their own page). </t>
+          <t xml:space="preserve">Specify different ways of displaying questions. 
+pages: show each question or field list on its own page.
+By default, all questions are shown on a single page.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>6</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>5</xdr:col>
+                <xdr:colOff>2</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="D1" authorId="0">
       <text>
@@ -197,16 +389,37 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Custom namespaces supported in the form.  `cht` must be included here to use the custom `instance::cht` columns on the survey sheet.</t>
+          <t xml:space="preserve">Specify the custom namespaces used in the form. For example: `cht=https://communityhealthtoolkit.org`.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>4</xdr:col>
+                <xdr:colOff>6</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>6</xdr:col>
+                <xdr:colOff>2</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="65">
   <si>
     <t xml:space="preserve">type</t>
   </si>
@@ -214,10 +427,10 @@
     <t xml:space="preserve">name</t>
   </si>
   <si>
-    <t xml:space="preserve">label::English (en)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hint::English (en)</t>
+    <t xml:space="preserve">label::en</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hint::en</t>
   </si>
   <si>
     <t xml:space="preserve">relevant</t>
@@ -286,9 +499,6 @@
     <t xml:space="preserve">description_conclusion</t>
   </si>
   <si>
-    <t xml:space="preserve">NO_LABEL</t>
-  </si>
-  <si>
     <t xml:space="preserve">${value_b} != “"</t>
   </si>
   <si>
@@ -332,21 +542,93 @@
   </si>
   <si>
     <t xml:space="preserve">cht=https://communityhealthtoolkit.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">survey_header_names</t>
+  </si>
+  <si>
+    <t xml:space="preserve">settings_header_names</t>
+  </si>
+  <si>
+    <t xml:space="preserve">allow_choice_duplicates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">audio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">choice_filter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constraint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constraint_message</t>
+  </si>
+  <si>
+    <t xml:space="preserve">default</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">image</t>
+  </si>
+  <si>
+    <t xml:space="preserve">instance::cht:duration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">instance::cht:unique_tel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">instance::db-doc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">instance::db-doc-ref</t>
+  </si>
+  <si>
+    <t xml:space="preserve">instance::tag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">instance::type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">parameters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">read_only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">repeat_count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">required_message</t>
+  </si>
+  <si>
+    <t xml:space="preserve">trigger</t>
+  </si>
+  <si>
+    <t xml:space="preserve">video</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
-    <numFmt numFmtId="166" formatCode="mm/dd/yy\ hh:mm\ AM/PM"/>
   </numFmts>
   <fonts count="7">
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
@@ -366,17 +648,16 @@
       <family val="0"/>
     </font>
     <font>
-      <b val="true"/>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="2"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
-      <family val="2"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
@@ -385,27 +666,15 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFCCCCCC"/>
-        <bgColor rgb="FFCCCCFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFAFD095"/>
-        <bgColor rgb="FFCCCCCC"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="6">
+  <borders count="1">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -413,71 +682,8 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="hair">
-        <color rgb="FF999999"/>
-      </left>
-      <right style="hair">
-        <color rgb="FF999999"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="hair">
-        <color rgb="FF999999"/>
-      </left>
-      <right style="hair">
-        <color rgb="FF999999"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF3465A4"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="hair">
-        <color rgb="FF999999"/>
-      </left>
-      <right style="hair">
-        <color rgb="FF999999"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FF3465A4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="hair">
-        <color rgb="FF999999"/>
-      </left>
-      <right style="hair">
-        <color rgb="FF999999"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF5B277D"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="hair">
-        <color rgb="FF999999"/>
-      </left>
-      <right style="hair">
-        <color rgb="FF999999"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FF5B277D"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="26">
+  <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -501,84 +707,253 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="1" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="3" borderId="0" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="12">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="15" builtinId="3"/>
     <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
     <cellStyle name="Currency" xfId="17" builtinId="4"/>
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="column_head" xfId="20"/>
-    <cellStyle name="column_head_i18n" xfId="21"/>
-    <cellStyle name="group_begin" xfId="22"/>
-    <cellStyle name="group_end" xfId="23"/>
-    <cellStyle name="repeat_begin" xfId="24"/>
-    <cellStyle name="repeat_end" xfId="25"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
+  <dxfs count="25">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <i val="1"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFAFD095"/>
+        </patternFill>
+      </fill>
       <border diagonalUp="false" diagonalDown="false">
-        <left style="hair">
-          <color rgb="FF999999"/>
+        <left style="thin">
+          <color rgb="FF808080"/>
         </left>
-        <right style="hair">
-          <color rgb="FF999999"/>
+        <right style="thin">
+          <color rgb="FF808080"/>
         </right>
+        <top/>
+        <bottom/>
+        <diagonal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <i val="1"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD3D3D3"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="false" diagonalDown="false">
+        <left style="thin">
+          <color rgb="FF808080"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF808080"/>
+        </right>
+        <top/>
+        <bottom/>
+        <diagonal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <i val="1"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCCCF0"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="false" diagonalDown="false">
+        <left style="thin">
+          <color rgb="FF808080"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF808080"/>
+        </right>
+        <top/>
+        <bottom/>
+        <diagonal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFAFD095"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="false" diagonalDown="false">
+        <left style="thin">
+          <color rgb="FF808080"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF808080"/>
+        </right>
+        <top/>
+        <bottom/>
+        <diagonal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD3D3D3"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="false" diagonalDown="false">
+        <left style="thin">
+          <color rgb="FF808080"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF808080"/>
+        </right>
+        <top/>
+        <bottom/>
+        <diagonal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCCCF0"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="false" diagonalDown="false">
+        <left style="thin">
+          <color rgb="FF808080"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF808080"/>
+        </right>
+        <top/>
+        <bottom/>
+        <diagonal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border diagonalUp="false" diagonalDown="false">
+        <left/>
+        <right/>
         <top style="medium">
-          <color rgb="FF3465A4"/>
+          <color rgb="FF0070C0"/>
         </top>
         <bottom/>
         <diagonal/>
@@ -586,29 +961,21 @@
     </dxf>
     <dxf>
       <border diagonalUp="false" diagonalDown="false">
-        <left style="hair">
-          <color rgb="FF999999"/>
-        </left>
-        <right style="hair">
-          <color rgb="FF999999"/>
-        </right>
+        <left/>
+        <right/>
         <top/>
         <bottom style="medium">
-          <color rgb="FF3465A4"/>
+          <color rgb="FF0070C0"/>
         </bottom>
         <diagonal/>
       </border>
     </dxf>
     <dxf>
       <border diagonalUp="false" diagonalDown="false">
-        <left style="hair">
-          <color rgb="FF999999"/>
-        </left>
-        <right style="hair">
-          <color rgb="FF999999"/>
-        </right>
+        <left/>
+        <right/>
         <top style="medium">
-          <color rgb="FF5B277D"/>
+          <color rgb="FF7030A0"/>
         </top>
         <bottom/>
         <diagonal/>
@@ -616,26 +983,98 @@
     </dxf>
     <dxf>
       <border diagonalUp="false" diagonalDown="false">
-        <left style="hair">
-          <color rgb="FF999999"/>
-        </left>
-        <right style="hair">
-          <color rgb="FF999999"/>
-        </right>
+        <left/>
+        <right/>
         <top/>
         <bottom style="medium">
-          <color rgb="FF5B277D"/>
+          <color rgb="FF7030A0"/>
         </bottom>
         <diagonal/>
       </border>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
-        <color rgb="FFCC0000"/>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <i val="1"/>
+        <sz val="10"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFCCCC"/>
+          <bgColor rgb="FFD3D3D3"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="false" diagonalDown="false">
+        <left style="thin">
+          <color rgb="FF808080"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF808080"/>
+        </right>
+        <top/>
+        <bottom/>
+        <diagonal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD3D3D3"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="false" diagonalDown="false">
+        <left style="thin">
+          <color rgb="FF808080"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF808080"/>
+        </right>
+        <top/>
+        <bottom/>
+        <diagonal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -644,7 +1083,7 @@
     <indexedColors>
       <rgbColor rgb="FF000000"/>
       <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFCC0000"/>
+      <rgbColor rgb="FFFF0000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -656,16 +1095,16 @@
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFCCCCCC"/>
+      <rgbColor rgb="FFD3D3D3"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF7030A0"/>
       <rgbColor rgb="FFFFFFCC"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF0070C0"/>
+      <rgbColor rgb="FFCCCCF0"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -681,22 +1120,22 @@
       <rgbColor rgb="FFAFD095"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCCCC"/>
+      <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF3465A4"/>
-      <rgbColor rgb="FF999999"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
       <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF5B277D"/>
+      <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
     </indexedColors>
   </colors>
@@ -711,37 +1150,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -814,8 +1253,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:BF14"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.93"/>
@@ -824,37 +1263,35 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="17.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="11.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="38.25"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="11.53"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="26" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="8" style="1" width="9"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="58" min="25" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="60" style="1" width="11.53"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -864,11 +1301,120 @@
       <c r="C3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
+      <c r="O3" s="2"/>
+      <c r="P3" s="2"/>
+      <c r="Q3" s="2"/>
+      <c r="R3" s="2"/>
+      <c r="S3" s="2"/>
+      <c r="T3" s="2"/>
+      <c r="U3" s="2"/>
+      <c r="V3" s="2"/>
+      <c r="W3" s="2"/>
+      <c r="X3" s="2"/>
+      <c r="Y3" s="2"/>
+      <c r="Z3" s="2"/>
+      <c r="AA3" s="2"/>
+      <c r="AB3" s="2"/>
+      <c r="AC3" s="2"/>
+      <c r="AD3" s="2"/>
+      <c r="AE3" s="2"/>
+      <c r="AF3" s="2"/>
+      <c r="AG3" s="2"/>
+      <c r="AH3" s="2"/>
+      <c r="AI3" s="2"/>
+      <c r="AJ3" s="2"/>
+      <c r="AK3" s="2"/>
+      <c r="AL3" s="2"/>
+      <c r="AM3" s="2"/>
+      <c r="AN3" s="2"/>
+      <c r="AO3" s="2"/>
+      <c r="AP3" s="2"/>
+      <c r="AQ3" s="2"/>
+      <c r="AR3" s="2"/>
+      <c r="AS3" s="2"/>
+      <c r="AT3" s="2"/>
+      <c r="AU3" s="2"/>
+      <c r="AV3" s="2"/>
+      <c r="AW3" s="2"/>
+      <c r="AX3" s="2"/>
+      <c r="AY3" s="2"/>
+      <c r="AZ3" s="2"/>
+      <c r="BA3" s="2"/>
+      <c r="BB3" s="2"/>
+      <c r="BC3" s="2"/>
+      <c r="BD3" s="2"/>
+      <c r="BE3" s="2"/>
+      <c r="BF3" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2"/>
+      <c r="O4" s="2"/>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2"/>
+      <c r="S4" s="2"/>
+      <c r="T4" s="2"/>
+      <c r="U4" s="2"/>
+      <c r="V4" s="2"/>
+      <c r="W4" s="2"/>
+      <c r="X4" s="2"/>
+      <c r="Y4" s="2"/>
+      <c r="Z4" s="2"/>
+      <c r="AA4" s="2"/>
+      <c r="AB4" s="2"/>
+      <c r="AC4" s="2"/>
+      <c r="AD4" s="2"/>
+      <c r="AE4" s="2"/>
+      <c r="AF4" s="2"/>
+      <c r="AG4" s="2"/>
+      <c r="AH4" s="2"/>
+      <c r="AI4" s="2"/>
+      <c r="AJ4" s="2"/>
+      <c r="AK4" s="2"/>
+      <c r="AL4" s="2"/>
+      <c r="AM4" s="2"/>
+      <c r="AN4" s="2"/>
+      <c r="AO4" s="2"/>
+      <c r="AP4" s="2"/>
+      <c r="AQ4" s="2"/>
+      <c r="AR4" s="2"/>
+      <c r="AS4" s="2"/>
+      <c r="AT4" s="2"/>
+      <c r="AU4" s="2"/>
+      <c r="AV4" s="2"/>
+      <c r="AW4" s="2"/>
+      <c r="AX4" s="2"/>
+      <c r="AY4" s="2"/>
+      <c r="AZ4" s="2"/>
+      <c r="BA4" s="2"/>
+      <c r="BB4" s="2"/>
+      <c r="BC4" s="2"/>
+      <c r="BD4" s="2"/>
+      <c r="BE4" s="2"/>
+      <c r="BF4" s="2"/>
+    </row>
+    <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -878,11 +1424,13 @@
       <c r="C5" s="1" t="s">
         <v>13</v>
       </c>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
       <c r="F5" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
@@ -893,7 +1441,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
         <v>17</v>
       </c>
@@ -904,7 +1452,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
         <v>20</v>
       </c>
@@ -915,7 +1463,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
         <v>17</v>
       </c>
@@ -926,106 +1474,197 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="E10" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E10" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="E11" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E11" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="E12" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E12" s="1" t="s">
+    </row>
+    <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
         <v>33</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <conditionalFormatting sqref="A2:H10000">
+  <conditionalFormatting sqref="A1:BF1">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>$A2="begin_group"</formula>
+      <formula>AND(A1&lt;&gt;"",COUNTIF($A$1:$BF$1,A1)&gt;1)</formula>
     </cfRule>
     <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>$A2="end_group"</formula>
+      <formula>AND(A1&lt;&gt;"",NOT(OR(A1="audio",LEFT(A1,7)="audio::",A1="constraint_message",LEFT(A1,20)="constraint_message::",A1="hint",LEFT(A1,6)="hint::",A1="image",LEFT(A1,7)="image::",A1="label",LEFT(A1,7)="label::",A1="required_message",LEFT(A1,18)="required_message::",A1="video",LEFT(A1,7)="video::")),NOT(NOT(ISERROR(MATCH(A1,{"appearance","instance::cht:duration","instance::cht:unique_tel","instance::db-doc","instance::db-doc-ref","instance::tag","instance::type","name","note","parameters","read_only","trigger","type"},0)))),NOT(NOT(ISERROR(MATCH(A1,{"calculation","choice_filter","constraint","default","relevant","repeat_count","required"},0)))))</formula>
     </cfRule>
     <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
-      <formula>$A2="begin_repeat"</formula>
+      <formula>AND(OR(A1="audio",LEFT(A1,7)="audio::",A1="constraint_message",LEFT(A1,20)="constraint_message::",A1="hint",LEFT(A1,6)="hint::",A1="image",LEFT(A1,7)="image::",A1="label",LEFT(A1,7)="label::",A1="required_message",LEFT(A1,18)="required_message::",A1="video",LEFT(A1,7)="video::"),COUNTA(A$3:A$1016)=0)</formula>
     </cfRule>
     <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
-      <formula>$A2="end_repeat"</formula>
+      <formula>AND(NOT(ISERROR(MATCH(A1,{"appearance","instance::cht:duration","instance::cht:unique_tel","instance::db-doc","instance::db-doc-ref","instance::tag","instance::type","name","note","parameters","read_only","trigger","type"},0))),COUNTA(A$3:A$1016)=0)</formula>
     </cfRule>
     <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
-      <formula>AND(ISBLANK($A2), NOT(ISBLANK(A2)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2:B10000">
-    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
-      <formula>AND(ISBLANK(B2), NOT(ISBLANK($A2)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C10000">
-    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
-      <formula>AND(ISBLANK(C2),NOT(OR(ISBLANK($A2),$A2="calculate")))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G10000">
-    <cfRule type="expression" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
-      <formula>AND($A2="calculate", ISBLANK(G2))</formula>
+      <formula>AND(NOT(ISERROR(MATCH(A1,{"calculation","choice_filter","constraint","default","relevant","repeat_count","required"},0))),COUNTA(A$3:A$1016)=0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
+      <formula>OR(A1="audio",LEFT(A1,7)="audio::",A1="constraint_message",LEFT(A1,20)="constraint_message::",A1="hint",LEFT(A1,6)="hint::",A1="image",LEFT(A1,7)="image::",A1="label",LEFT(A1,7)="label::",A1="required_message",LEFT(A1,18)="required_message::",A1="video",LEFT(A1,7)="video::")</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+      <formula>NOT(ISERROR(MATCH(A1,{"appearance","instance::cht:duration","instance::cht:unique_tel","instance::db-doc","instance::db-doc-ref","instance::tag","instance::type","name","note","parameters","read_only","trigger","type"},0)))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+      <formula>NOT(ISERROR(MATCH(A1,{"calculation","choice_filter","constraint","default","relevant","repeat_count","required"},0)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A3:A1016">
+    <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+      <formula>AND(A3&lt;&gt;"",NOT(OR(NOT(ISERROR(MATCH(A3,{"acknowledge","audio","begin_group","begin_repeat","calculate","date","datetime","decimal","end","end_group","end_repeat","file","geopoint","geoshape","geotrace","hidden","image","integer","note","range","rank","start","text","time","today","video"},0))),0,0)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B1016">
+    <cfRule type="expression" priority="11" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+      <formula>AND(A3&lt;&gt;"",B3="")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C3:C1016">
+    <cfRule type="expression" priority="12" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+      <formula>AND(OR(NOT(ISERROR(MATCH(A3,{"acknowledge","audio","date","datetime","decimal","file","geopoint","geoshape","geotrace","image","integer","note","range","rank","text","time","video"},0))),LEFT(A3,11)="select_one ",LEFT(A3,16)="select_multiple "),C3="")</formula>
+    </cfRule>
+    <cfRule type="expression" priority="13" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+      <formula>AND(C3&lt;&gt;"",NOT(ISERROR(MATCH(A3,{"calculate","end","end_group","end_repeat","hidden","start","today"},0))))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="14" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
+      <formula>OR(C3="NO_LABEL",C3="DELETE_THIS_LINE")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G3:G1016">
+    <cfRule type="expression" priority="15" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+      <formula>AND(A3="calculate",G3="")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A3:BF1016">
+    <cfRule type="expression" priority="16" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+      <formula>AND($A3="begin_group",A$1&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A3:BF1016">
+    <cfRule type="expression" priority="17" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+      <formula>AND($A3="end_group",A$1&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A3:BF1016">
+    <cfRule type="expression" priority="18" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
+      <formula>AND($A3="begin_repeat",A$1&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A3:BF1016">
+    <cfRule type="expression" priority="19" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
+      <formula>AND($A3="end_repeat",A$1&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A3:BF1016">
+    <cfRule type="expression" priority="20" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
+      <formula>AND(A3&lt;&gt;"",A$1="")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2">
+    <cfRule type="expression" priority="21" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+      <formula>AND(A2&lt;&gt;"",NOT(OR(NOT(ISERROR(MATCH(A2,{"acknowledge","audio","begin_group","begin_repeat","calculate","date","datetime","decimal","end","end_group","end_repeat","file","geopoint","geoshape","geotrace","hidden","image","integer","note","range","rank","start","text","time","today","video"},0))),0,0)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2">
+    <cfRule type="expression" priority="22" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+      <formula>AND(A2&lt;&gt;"",B2="")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C2">
+    <cfRule type="expression" priority="23" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+      <formula>AND(OR(NOT(ISERROR(MATCH(A2,{"acknowledge","audio","date","datetime","decimal","file","geopoint","geoshape","geotrace","image","integer","note","range","rank","text","time","video"},0))),LEFT(A2,11)="select_one ",LEFT(A2,16)="select_multiple "),C2="")</formula>
+    </cfRule>
+    <cfRule type="expression" priority="24" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+      <formula>AND(C2&lt;&gt;"",NOT(ISERROR(MATCH(A2,{"calculate","end","end_group","end_repeat","hidden","start","today"},0))))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="25" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
+      <formula>OR(C2="NO_LABEL",C2="DELETE_THIS_LINE")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2">
+    <cfRule type="expression" priority="26" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+      <formula>AND(A2="calculate",G2="")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:BF2">
+    <cfRule type="expression" priority="27" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+      <formula>AND($A2="begin_group",A$1&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:BF2">
+    <cfRule type="expression" priority="28" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+      <formula>AND($A2="end_group",A$1&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:BF2">
+    <cfRule type="expression" priority="29" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
+      <formula>AND($A2="begin_repeat",A$1&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:BF2">
+    <cfRule type="expression" priority="30" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
+      <formula>AND($A2="end_repeat",A$1&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:BF2">
+    <cfRule type="expression" priority="31" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
+      <formula>AND(A2&lt;&gt;"",A$1="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" error="If configuring a select, ensure your list name matches a list from the choices sheet." errorStyle="information" operator="equal" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="A1" type="none">
-      <formula1>0</formula1>
+    <dataValidation allowBlank="true" error="For translatable columns, you can append &quot;::&lt;lang&gt;&quot; to the column name (e.g., label::en)." errorStyle="information" errorTitle="Column warning" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A1:BF1" type="list">
+      <formula1>chtx!$A$2:$A$28</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="If configuring a select, ensure your list name matches a list from the choices sheet." errorStyle="information" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A2:A1014" type="list">
-      <formula1>"begin_group,end_group,note,calculate,text,integer,decimal,select_one list_name,select_multiple list_name,date,time,datetime,begin_repeat,end_repeat,geopoint,geotrace,geoshape,start-geopoint,range,image,audio,video,file,rank,acknowledge,start,end,today"</formula1>
+    <dataValidation allowBlank="true" error="If configuring a select, ensure your list name matches a list from the choices sheet." errorStyle="information" errorTitle="Type warning" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A2:A1014" type="list">
+      <formula1>"acknowledge,audio,begin_group,begin_repeat,calculate,date,datetime,decimal,end,end_group,end_repeat,file,geopoint,geoshape,geotrace,hidden,image,integer,note,range,rank,select_multiple list_name,select_one list_name,start,text,time,today,video"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -1049,50 +1688,262 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="5" width="17.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="5" width="16.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="5" width="32.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="3" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="32.61"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
+    <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="C1" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="D1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D1" s="6" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
+      <c r="B2" s="1" t="str">
+        <f aca="true">TEXT(NOW(), "yyyymmddhhmmss")</f>
+        <v>20260618172109</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B2" s="7" t="str">
-        <f aca="true">TEXT(NOW(), "yyyymmddhhmmss")</f>
-        <v>20260114091928</v>
-      </c>
-      <c r="C2" s="5" t="s">
+      <c r="D2" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D2" s="5" t="s">
-        <v>41</v>
-      </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A1:BC1">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
+      <formula>AND(A1&lt;&gt;"",COUNTIF($A$1:$BC$1,A1)&gt;1)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
+      <formula>AND(A1&lt;&gt;"",NOT(NOT(ISERROR(MATCH(A1,{"allow_choice_duplicates","form_title","namespaces","style","version"},0)))))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="21">
+      <formula>AND(A1&lt;&gt;"",COUNTA(A$2:A$1002)=0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="22">
+      <formula>NOT(ISERROR(MATCH(A1,{"allow_choice_duplicates","form_title","namespaces","style","version"},0)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C2:C1002">
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="23">
+      <formula>AND(C2&lt;&gt;"",C2&lt;&gt;"pages")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:BC1002">
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="24">
+      <formula>AND(A2&lt;&gt;"",A$1="")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation allowBlank="true" error="Unexpected column name." errorStyle="information" errorTitle="Column warning" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A1:BC1" type="list">
+      <formula1>chtx!$C$2:$C$6</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" error="This column only accepts &quot;pages&quot; or an empty value." errorStyle="stop" errorTitle="Invalid value" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C2:C1002" type="list">
+      <formula1>",pages"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;A</oddHeader>
     <oddFooter>&amp;CPage &amp;P</oddFooter>
   </headerFooter>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C28"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
chore: format all forms with chtoolbox (#37)
</commit_message>
<xml_diff>
--- a/basic-forms/forms/app/comparing_values.xlsx
+++ b/basic-forms/forms/app/comparing_values.xlsx
@@ -1,8 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <fileVersion appName="Calc" lowestEdited="5"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
@@ -10,20 +10,21 @@
   <sheets>
     <sheet name="survey" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="settings" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="chtx" sheetId="3" state="hidden" r:id="rId5"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
+      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
   <authors>
-    <author>Unknown Author</author>
+    <author>Author</author>
   </authors>
   <commentList>
     <comment ref="A1" authorId="0">
@@ -35,20 +36,30 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">Determines what kinds of values are allowed and how the field is displayed. For certain types, further customization is possible using the appearance and parameters columns.
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF0000FF"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">https://docs.getodk.org/form-question-types/
-</t>
+https://docs.getodk.org/form-question-types/</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>6</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>2</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="B1" authorId="0">
       <text>
@@ -61,6 +72,27 @@
           <t xml:space="preserve">Variable name. It may not contain spaces and must start with a letter or underscore. You should use a short, descriptive name and can use underscores to separate words. For example: date_of_birth.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>2</xdr:col>
+                <xdr:colOff>6</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>4</xdr:col>
+                <xdr:colOff>2</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="C1" authorId="0">
       <text>
@@ -74,6 +106,27 @@
 Can be translated.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>6</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>5</xdr:col>
+                <xdr:colOff>2</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="D1" authorId="0">
       <text>
@@ -87,6 +140,27 @@
 Can be translated.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>4</xdr:col>
+                <xdr:colOff>6</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>6</xdr:col>
+                <xdr:colOff>2</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="E1" authorId="0">
       <text>
@@ -97,9 +171,30 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">An expression that determines whether a question will be displayed to a user or not. Lets you define branching or skip logic. 
-https://docs.getodk.org/form-logic/#conditionally-showing-questions</t>
+See the Relevance tab for examples.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>5</xdr:col>
+                <xdr:colOff>6</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>7</xdr:col>
+                <xdr:colOff>2</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="F1" authorId="0">
       <text>
@@ -113,6 +208,27 @@
 These can be specific to the field type.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>6</xdr:col>
+                <xdr:colOff>6</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>8</xdr:col>
+                <xdr:colOff>21</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="G1" authorId="0">
       <text>
@@ -123,32 +239,41 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">An expression that will be evaluated to determine the value of the field.
-⚠️ Expressions may be re-evaluated at any time. 
-To limit when expressions are evaluated, for example to specify dynamic defaults use the once() function. 
+Expressions may be re-evaluated at any time. Question types with calculations should be marked as read-only. Otherwise, a user-provided value may be replaced by a calculated one.
+To limit when expressions are evaluated, for example to specify dynamic defaults, use the trigger column or the once() function. 
 https://docs.getodk.org/form-logic/#when-expressions-are-evaluated</t>
         </r>
       </text>
-    </comment>
-    <comment ref="H1" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Can include a human-friendly note to describe the row. This will be ignored by all ODK tools.</t>
-        </r>
-      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>7</xdr:col>
+                <xdr:colOff>6</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>9</xdr:col>
+                <xdr:colOff>21</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
   <authors>
-    <author>Unknown Author</author>
+    <author>Author</author>
   </authors>
   <commentList>
     <comment ref="A1" authorId="0">
@@ -163,6 +288,27 @@
 https://docs.getodk.org/xlsform/#the-settings-sheet</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>6</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>2</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="B1" authorId="0">
       <text>
@@ -173,9 +319,32 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">The unique version code that identifies the current state of the form. A common convention is to use a format like yyyymmddrr. For example, 2017021501 is the 1st revision from Feb 15th, 2017.
-By default, this template uses a formula to create a date-based version that will update automatically.</t>
+A formula can be used to update the version automatically: `=TEXT(NOW(), "yyyymmddhhmmss")`
+This `version` is recorded in the form xml and is primarily useful for determining which version of the xlsform was used to produce the xml. A separate `form_version` property is generated for each form when it is uploaded to the CHT server. This is the version set on report docs produced by the form.
+https://docs.communityhealthtoolkit.org/building/forms/versioning/</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>2</xdr:col>
+                <xdr:colOff>6</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>4</xdr:col>
+                <xdr:colOff>2</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="C1" authorId="0">
       <text>
@@ -185,9 +354,32 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Set to ‘pages’ to indicate that groups with the `field-list` appearance represent separate form pages (and all other questions will be shown on their own page). </t>
+          <t xml:space="preserve">Specify different ways of displaying questions. 
+pages: show each question or field list on its own page.
+By default, all questions are shown on a single page.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>6</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>5</xdr:col>
+                <xdr:colOff>2</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
     <comment ref="D1" authorId="0">
       <text>
@@ -197,16 +389,37 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Custom namespaces supported in the form.  `cht` must be included here to use the custom `instance::cht` columns on the survey sheet.</t>
+          <t xml:space="preserve">Specify the custom namespaces used in the form. For example: `cht=https://communityhealthtoolkit.org`.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>4</xdr:col>
+                <xdr:colOff>6</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>14</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>6</xdr:col>
+                <xdr:colOff>2</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>16</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="65">
   <si>
     <t xml:space="preserve">type</t>
   </si>
@@ -214,10 +427,10 @@
     <t xml:space="preserve">name</t>
   </si>
   <si>
-    <t xml:space="preserve">label::English (en)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hint::English (en)</t>
+    <t xml:space="preserve">label::en</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hint::en</t>
   </si>
   <si>
     <t xml:space="preserve">relevant</t>
@@ -286,9 +499,6 @@
     <t xml:space="preserve">description_conclusion</t>
   </si>
   <si>
-    <t xml:space="preserve">NO_LABEL</t>
-  </si>
-  <si>
     <t xml:space="preserve">${value_b} != “"</t>
   </si>
   <si>
@@ -332,21 +542,93 @@
   </si>
   <si>
     <t xml:space="preserve">cht=https://communityhealthtoolkit.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">survey_header_names</t>
+  </si>
+  <si>
+    <t xml:space="preserve">settings_header_names</t>
+  </si>
+  <si>
+    <t xml:space="preserve">allow_choice_duplicates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">audio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">choice_filter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constraint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">constraint_message</t>
+  </si>
+  <si>
+    <t xml:space="preserve">default</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">image</t>
+  </si>
+  <si>
+    <t xml:space="preserve">instance::cht:duration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">instance::cht:unique_tel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">instance::db-doc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">instance::db-doc-ref</t>
+  </si>
+  <si>
+    <t xml:space="preserve">instance::tag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">instance::type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">parameters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">read_only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">repeat_count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">required_message</t>
+  </si>
+  <si>
+    <t xml:space="preserve">trigger</t>
+  </si>
+  <si>
+    <t xml:space="preserve">video</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
-    <numFmt numFmtId="166" formatCode="mm/dd/yy\ hh:mm\ AM/PM"/>
   </numFmts>
   <fonts count="7">
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
@@ -366,17 +648,16 @@
       <family val="0"/>
     </font>
     <font>
-      <b val="true"/>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="2"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
-      <family val="2"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
@@ -385,27 +666,15 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFCCCCCC"/>
-        <bgColor rgb="FFCCCCFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFAFD095"/>
-        <bgColor rgb="FFCCCCCC"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="6">
+  <borders count="1">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -413,71 +682,8 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="hair">
-        <color rgb="FF999999"/>
-      </left>
-      <right style="hair">
-        <color rgb="FF999999"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="hair">
-        <color rgb="FF999999"/>
-      </left>
-      <right style="hair">
-        <color rgb="FF999999"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF3465A4"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="hair">
-        <color rgb="FF999999"/>
-      </left>
-      <right style="hair">
-        <color rgb="FF999999"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FF3465A4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="hair">
-        <color rgb="FF999999"/>
-      </left>
-      <right style="hair">
-        <color rgb="FF999999"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF5B277D"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="hair">
-        <color rgb="FF999999"/>
-      </left>
-      <right style="hair">
-        <color rgb="FF999999"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FF5B277D"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="26">
+  <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -501,84 +707,253 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="1" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="3" borderId="0" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="12">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="15" builtinId="3"/>
     <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
     <cellStyle name="Currency" xfId="17" builtinId="4"/>
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="column_head" xfId="20"/>
-    <cellStyle name="column_head_i18n" xfId="21"/>
-    <cellStyle name="group_begin" xfId="22"/>
-    <cellStyle name="group_end" xfId="23"/>
-    <cellStyle name="repeat_begin" xfId="24"/>
-    <cellStyle name="repeat_end" xfId="25"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
+  <dxfs count="25">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <i val="1"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFAFD095"/>
+        </patternFill>
+      </fill>
       <border diagonalUp="false" diagonalDown="false">
-        <left style="hair">
-          <color rgb="FF999999"/>
+        <left style="thin">
+          <color rgb="FF808080"/>
         </left>
-        <right style="hair">
-          <color rgb="FF999999"/>
+        <right style="thin">
+          <color rgb="FF808080"/>
         </right>
+        <top/>
+        <bottom/>
+        <diagonal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <i val="1"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD3D3D3"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="false" diagonalDown="false">
+        <left style="thin">
+          <color rgb="FF808080"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF808080"/>
+        </right>
+        <top/>
+        <bottom/>
+        <diagonal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <i val="1"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCCCF0"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="false" diagonalDown="false">
+        <left style="thin">
+          <color rgb="FF808080"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF808080"/>
+        </right>
+        <top/>
+        <bottom/>
+        <diagonal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFAFD095"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="false" diagonalDown="false">
+        <left style="thin">
+          <color rgb="FF808080"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF808080"/>
+        </right>
+        <top/>
+        <bottom/>
+        <diagonal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD3D3D3"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="false" diagonalDown="false">
+        <left style="thin">
+          <color rgb="FF808080"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF808080"/>
+        </right>
+        <top/>
+        <bottom/>
+        <diagonal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCCCF0"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="false" diagonalDown="false">
+        <left style="thin">
+          <color rgb="FF808080"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF808080"/>
+        </right>
+        <top/>
+        <bottom/>
+        <diagonal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border diagonalUp="false" diagonalDown="false">
+        <left/>
+        <right/>
         <top style="medium">
-          <color rgb="FF3465A4"/>
+          <color rgb="FF0070C0"/>
         </top>
         <bottom/>
         <diagonal/>
@@ -586,29 +961,21 @@
     </dxf>
     <dxf>
       <border diagonalUp="false" diagonalDown="false">
-        <left style="hair">
-          <color rgb="FF999999"/>
-        </left>
-        <right style="hair">
-          <color rgb="FF999999"/>
-        </right>
+        <left/>
+        <right/>
         <top/>
         <bottom style="medium">
-          <color rgb="FF3465A4"/>
+          <color rgb="FF0070C0"/>
         </bottom>
         <diagonal/>
       </border>
     </dxf>
     <dxf>
       <border diagonalUp="false" diagonalDown="false">
-        <left style="hair">
-          <color rgb="FF999999"/>
-        </left>
-        <right style="hair">
-          <color rgb="FF999999"/>
-        </right>
+        <left/>
+        <right/>
         <top style="medium">
-          <color rgb="FF5B277D"/>
+          <color rgb="FF7030A0"/>
         </top>
         <bottom/>
         <diagonal/>
@@ -616,26 +983,98 @@
     </dxf>
     <dxf>
       <border diagonalUp="false" diagonalDown="false">
-        <left style="hair">
-          <color rgb="FF999999"/>
-        </left>
-        <right style="hair">
-          <color rgb="FF999999"/>
-        </right>
+        <left/>
+        <right/>
         <top/>
         <bottom style="medium">
-          <color rgb="FF5B277D"/>
+          <color rgb="FF7030A0"/>
         </bottom>
         <diagonal/>
       </border>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
-        <color rgb="FFCC0000"/>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <i val="1"/>
+        <sz val="10"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFCCCC"/>
+          <bgColor rgb="FFD3D3D3"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="false" diagonalDown="false">
+        <left style="thin">
+          <color rgb="FF808080"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF808080"/>
+        </right>
+        <top/>
+        <bottom/>
+        <diagonal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD3D3D3"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="false" diagonalDown="false">
+        <left style="thin">
+          <color rgb="FF808080"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF808080"/>
+        </right>
+        <top/>
+        <bottom/>
+        <diagonal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -644,7 +1083,7 @@
     <indexedColors>
       <rgbColor rgb="FF000000"/>
       <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFCC0000"/>
+      <rgbColor rgb="FFFF0000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -656,16 +1095,16 @@
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFCCCCCC"/>
+      <rgbColor rgb="FFD3D3D3"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF7030A0"/>
       <rgbColor rgb="FFFFFFCC"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF0070C0"/>
+      <rgbColor rgb="FFCCCCF0"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -681,22 +1120,22 @@
       <rgbColor rgb="FFAFD095"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCCCC"/>
+      <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF3465A4"/>
-      <rgbColor rgb="FF999999"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
       <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF5B277D"/>
+      <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
     </indexedColors>
   </colors>
@@ -711,37 +1150,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -814,8 +1253,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:BF14"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.93"/>
@@ -824,37 +1263,35 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="17.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="11.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="38.25"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="11.53"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="26" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="8" style="1" width="9"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="58" min="25" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="60" style="1" width="11.53"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -864,11 +1301,120 @@
       <c r="C3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
+      <c r="O3" s="2"/>
+      <c r="P3" s="2"/>
+      <c r="Q3" s="2"/>
+      <c r="R3" s="2"/>
+      <c r="S3" s="2"/>
+      <c r="T3" s="2"/>
+      <c r="U3" s="2"/>
+      <c r="V3" s="2"/>
+      <c r="W3" s="2"/>
+      <c r="X3" s="2"/>
+      <c r="Y3" s="2"/>
+      <c r="Z3" s="2"/>
+      <c r="AA3" s="2"/>
+      <c r="AB3" s="2"/>
+      <c r="AC3" s="2"/>
+      <c r="AD3" s="2"/>
+      <c r="AE3" s="2"/>
+      <c r="AF3" s="2"/>
+      <c r="AG3" s="2"/>
+      <c r="AH3" s="2"/>
+      <c r="AI3" s="2"/>
+      <c r="AJ3" s="2"/>
+      <c r="AK3" s="2"/>
+      <c r="AL3" s="2"/>
+      <c r="AM3" s="2"/>
+      <c r="AN3" s="2"/>
+      <c r="AO3" s="2"/>
+      <c r="AP3" s="2"/>
+      <c r="AQ3" s="2"/>
+      <c r="AR3" s="2"/>
+      <c r="AS3" s="2"/>
+      <c r="AT3" s="2"/>
+      <c r="AU3" s="2"/>
+      <c r="AV3" s="2"/>
+      <c r="AW3" s="2"/>
+      <c r="AX3" s="2"/>
+      <c r="AY3" s="2"/>
+      <c r="AZ3" s="2"/>
+      <c r="BA3" s="2"/>
+      <c r="BB3" s="2"/>
+      <c r="BC3" s="2"/>
+      <c r="BD3" s="2"/>
+      <c r="BE3" s="2"/>
+      <c r="BF3" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2"/>
+      <c r="O4" s="2"/>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2"/>
+      <c r="S4" s="2"/>
+      <c r="T4" s="2"/>
+      <c r="U4" s="2"/>
+      <c r="V4" s="2"/>
+      <c r="W4" s="2"/>
+      <c r="X4" s="2"/>
+      <c r="Y4" s="2"/>
+      <c r="Z4" s="2"/>
+      <c r="AA4" s="2"/>
+      <c r="AB4" s="2"/>
+      <c r="AC4" s="2"/>
+      <c r="AD4" s="2"/>
+      <c r="AE4" s="2"/>
+      <c r="AF4" s="2"/>
+      <c r="AG4" s="2"/>
+      <c r="AH4" s="2"/>
+      <c r="AI4" s="2"/>
+      <c r="AJ4" s="2"/>
+      <c r="AK4" s="2"/>
+      <c r="AL4" s="2"/>
+      <c r="AM4" s="2"/>
+      <c r="AN4" s="2"/>
+      <c r="AO4" s="2"/>
+      <c r="AP4" s="2"/>
+      <c r="AQ4" s="2"/>
+      <c r="AR4" s="2"/>
+      <c r="AS4" s="2"/>
+      <c r="AT4" s="2"/>
+      <c r="AU4" s="2"/>
+      <c r="AV4" s="2"/>
+      <c r="AW4" s="2"/>
+      <c r="AX4" s="2"/>
+      <c r="AY4" s="2"/>
+      <c r="AZ4" s="2"/>
+      <c r="BA4" s="2"/>
+      <c r="BB4" s="2"/>
+      <c r="BC4" s="2"/>
+      <c r="BD4" s="2"/>
+      <c r="BE4" s="2"/>
+      <c r="BF4" s="2"/>
+    </row>
+    <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -878,11 +1424,13 @@
       <c r="C5" s="1" t="s">
         <v>13</v>
       </c>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
       <c r="F5" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
@@ -893,7 +1441,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
         <v>17</v>
       </c>
@@ -904,7 +1452,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
         <v>20</v>
       </c>
@@ -915,7 +1463,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
         <v>17</v>
       </c>
@@ -926,106 +1474,197 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="E10" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E10" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="E11" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E11" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="E12" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E12" s="1" t="s">
+    </row>
+    <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
         <v>33</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <conditionalFormatting sqref="A2:H10000">
+  <conditionalFormatting sqref="A1:BF1">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>$A2="begin_group"</formula>
+      <formula>AND(A1&lt;&gt;"",COUNTIF($A$1:$BF$1,A1)&gt;1)</formula>
     </cfRule>
     <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>$A2="end_group"</formula>
+      <formula>AND(A1&lt;&gt;"",NOT(OR(A1="audio",LEFT(A1,7)="audio::",A1="constraint_message",LEFT(A1,20)="constraint_message::",A1="hint",LEFT(A1,6)="hint::",A1="image",LEFT(A1,7)="image::",A1="label",LEFT(A1,7)="label::",A1="required_message",LEFT(A1,18)="required_message::",A1="video",LEFT(A1,7)="video::")),NOT(NOT(ISERROR(MATCH(A1,{"appearance","instance::cht:duration","instance::cht:unique_tel","instance::db-doc","instance::db-doc-ref","instance::tag","instance::type","name","note","parameters","read_only","trigger","type"},0)))),NOT(NOT(ISERROR(MATCH(A1,{"calculation","choice_filter","constraint","default","relevant","repeat_count","required"},0)))))</formula>
     </cfRule>
     <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
-      <formula>$A2="begin_repeat"</formula>
+      <formula>AND(OR(A1="audio",LEFT(A1,7)="audio::",A1="constraint_message",LEFT(A1,20)="constraint_message::",A1="hint",LEFT(A1,6)="hint::",A1="image",LEFT(A1,7)="image::",A1="label",LEFT(A1,7)="label::",A1="required_message",LEFT(A1,18)="required_message::",A1="video",LEFT(A1,7)="video::"),COUNTA(A$3:A$1016)=0)</formula>
     </cfRule>
     <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
-      <formula>$A2="end_repeat"</formula>
+      <formula>AND(NOT(ISERROR(MATCH(A1,{"appearance","instance::cht:duration","instance::cht:unique_tel","instance::db-doc","instance::db-doc-ref","instance::tag","instance::type","name","note","parameters","read_only","trigger","type"},0))),COUNTA(A$3:A$1016)=0)</formula>
     </cfRule>
     <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
-      <formula>AND(ISBLANK($A2), NOT(ISBLANK(A2)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2:B10000">
-    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
-      <formula>AND(ISBLANK(B2), NOT(ISBLANK($A2)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C10000">
-    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
-      <formula>AND(ISBLANK(C2),NOT(OR(ISBLANK($A2),$A2="calculate")))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G10000">
-    <cfRule type="expression" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
-      <formula>AND($A2="calculate", ISBLANK(G2))</formula>
+      <formula>AND(NOT(ISERROR(MATCH(A1,{"calculation","choice_filter","constraint","default","relevant","repeat_count","required"},0))),COUNTA(A$3:A$1016)=0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
+      <formula>OR(A1="audio",LEFT(A1,7)="audio::",A1="constraint_message",LEFT(A1,20)="constraint_message::",A1="hint",LEFT(A1,6)="hint::",A1="image",LEFT(A1,7)="image::",A1="label",LEFT(A1,7)="label::",A1="required_message",LEFT(A1,18)="required_message::",A1="video",LEFT(A1,7)="video::")</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+      <formula>NOT(ISERROR(MATCH(A1,{"appearance","instance::cht:duration","instance::cht:unique_tel","instance::db-doc","instance::db-doc-ref","instance::tag","instance::type","name","note","parameters","read_only","trigger","type"},0)))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+      <formula>NOT(ISERROR(MATCH(A1,{"calculation","choice_filter","constraint","default","relevant","repeat_count","required"},0)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A3:A1016">
+    <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+      <formula>AND(A3&lt;&gt;"",NOT(OR(NOT(ISERROR(MATCH(A3,{"acknowledge","audio","begin_group","begin_repeat","calculate","date","datetime","decimal","end","end_group","end_repeat","file","geopoint","geoshape","geotrace","hidden","image","integer","note","range","rank","start","text","time","today","video"},0))),0,0)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B1016">
+    <cfRule type="expression" priority="11" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+      <formula>AND(A3&lt;&gt;"",B3="")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C3:C1016">
+    <cfRule type="expression" priority="12" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+      <formula>AND(OR(NOT(ISERROR(MATCH(A3,{"acknowledge","audio","date","datetime","decimal","file","geopoint","geoshape","geotrace","image","integer","note","range","rank","text","time","video"},0))),LEFT(A3,11)="select_one ",LEFT(A3,16)="select_multiple "),C3="")</formula>
+    </cfRule>
+    <cfRule type="expression" priority="13" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+      <formula>AND(C3&lt;&gt;"",NOT(ISERROR(MATCH(A3,{"calculate","end","end_group","end_repeat","hidden","start","today"},0))))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="14" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
+      <formula>OR(C3="NO_LABEL",C3="DELETE_THIS_LINE")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G3:G1016">
+    <cfRule type="expression" priority="15" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+      <formula>AND(A3="calculate",G3="")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A3:BF1016">
+    <cfRule type="expression" priority="16" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+      <formula>AND($A3="begin_group",A$1&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A3:BF1016">
+    <cfRule type="expression" priority="17" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+      <formula>AND($A3="end_group",A$1&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A3:BF1016">
+    <cfRule type="expression" priority="18" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
+      <formula>AND($A3="begin_repeat",A$1&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A3:BF1016">
+    <cfRule type="expression" priority="19" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
+      <formula>AND($A3="end_repeat",A$1&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A3:BF1016">
+    <cfRule type="expression" priority="20" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
+      <formula>AND(A3&lt;&gt;"",A$1="")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2">
+    <cfRule type="expression" priority="21" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+      <formula>AND(A2&lt;&gt;"",NOT(OR(NOT(ISERROR(MATCH(A2,{"acknowledge","audio","begin_group","begin_repeat","calculate","date","datetime","decimal","end","end_group","end_repeat","file","geopoint","geoshape","geotrace","hidden","image","integer","note","range","rank","start","text","time","today","video"},0))),0,0)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2">
+    <cfRule type="expression" priority="22" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+      <formula>AND(A2&lt;&gt;"",B2="")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C2">
+    <cfRule type="expression" priority="23" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+      <formula>AND(OR(NOT(ISERROR(MATCH(A2,{"acknowledge","audio","date","datetime","decimal","file","geopoint","geoshape","geotrace","image","integer","note","range","rank","text","time","video"},0))),LEFT(A2,11)="select_one ",LEFT(A2,16)="select_multiple "),C2="")</formula>
+    </cfRule>
+    <cfRule type="expression" priority="24" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+      <formula>AND(C2&lt;&gt;"",NOT(ISERROR(MATCH(A2,{"calculate","end","end_group","end_repeat","hidden","start","today"},0))))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="25" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
+      <formula>OR(C2="NO_LABEL",C2="DELETE_THIS_LINE")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2">
+    <cfRule type="expression" priority="26" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+      <formula>AND(A2="calculate",G2="")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:BF2">
+    <cfRule type="expression" priority="27" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+      <formula>AND($A2="begin_group",A$1&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:BF2">
+    <cfRule type="expression" priority="28" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+      <formula>AND($A2="end_group",A$1&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:BF2">
+    <cfRule type="expression" priority="29" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
+      <formula>AND($A2="begin_repeat",A$1&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:BF2">
+    <cfRule type="expression" priority="30" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
+      <formula>AND($A2="end_repeat",A$1&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:BF2">
+    <cfRule type="expression" priority="31" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
+      <formula>AND(A2&lt;&gt;"",A$1="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" error="If configuring a select, ensure your list name matches a list from the choices sheet." errorStyle="information" operator="equal" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="A1" type="none">
-      <formula1>0</formula1>
+    <dataValidation allowBlank="true" error="For translatable columns, you can append &quot;::&lt;lang&gt;&quot; to the column name (e.g., label::en)." errorStyle="information" errorTitle="Column warning" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A1:BF1" type="list">
+      <formula1>chtx!$A$2:$A$28</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="If configuring a select, ensure your list name matches a list from the choices sheet." errorStyle="information" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A2:A1014" type="list">
-      <formula1>"begin_group,end_group,note,calculate,text,integer,decimal,select_one list_name,select_multiple list_name,date,time,datetime,begin_repeat,end_repeat,geopoint,geotrace,geoshape,start-geopoint,range,image,audio,video,file,rank,acknowledge,start,end,today"</formula1>
+    <dataValidation allowBlank="true" error="If configuring a select, ensure your list name matches a list from the choices sheet." errorStyle="information" errorTitle="Type warning" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A2:A1014" type="list">
+      <formula1>"acknowledge,audio,begin_group,begin_repeat,calculate,date,datetime,decimal,end,end_group,end_repeat,file,geopoint,geoshape,geotrace,hidden,image,integer,note,range,rank,select_multiple list_name,select_one list_name,start,text,time,today,video"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -1049,50 +1688,262 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="5" width="17.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="5" width="16.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="5" width="32.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="3" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="32.61"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
+    <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="C1" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="D1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D1" s="6" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
+      <c r="B2" s="1" t="str">
+        <f aca="true">TEXT(NOW(), "yyyymmddhhmmss")</f>
+        <v>20260618172109</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B2" s="7" t="str">
-        <f aca="true">TEXT(NOW(), "yyyymmddhhmmss")</f>
-        <v>20260114091928</v>
-      </c>
-      <c r="C2" s="5" t="s">
+      <c r="D2" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D2" s="5" t="s">
-        <v>41</v>
-      </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A1:BC1">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
+      <formula>AND(A1&lt;&gt;"",COUNTIF($A$1:$BC$1,A1)&gt;1)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
+      <formula>AND(A1&lt;&gt;"",NOT(NOT(ISERROR(MATCH(A1,{"allow_choice_duplicates","form_title","namespaces","style","version"},0)))))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="21">
+      <formula>AND(A1&lt;&gt;"",COUNTA(A$2:A$1002)=0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="22">
+      <formula>NOT(ISERROR(MATCH(A1,{"allow_choice_duplicates","form_title","namespaces","style","version"},0)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C2:C1002">
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="23">
+      <formula>AND(C2&lt;&gt;"",C2&lt;&gt;"pages")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:BC1002">
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="24">
+      <formula>AND(A2&lt;&gt;"",A$1="")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation allowBlank="true" error="Unexpected column name." errorStyle="information" errorTitle="Column warning" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A1:BC1" type="list">
+      <formula1>chtx!$C$2:$C$6</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" error="This column only accepts &quot;pages&quot; or an empty value." errorStyle="stop" errorTitle="Invalid value" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C2:C1002" type="list">
+      <formula1>",pages"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;A</oddHeader>
     <oddFooter>&amp;CPage &amp;P</oddFooter>
   </headerFooter>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C28"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>